<commit_message>
added output token count and throughput to metrics
</commit_message>
<xml_diff>
--- a/res/efficiency/pet-md/ollama-L3.3-MS-Nevoria-70b-Q4_K_S/2025-02-15_05-49-12/stats_by_iteration-L3.3-MS-Nevoria-70b-Q4_K_S.xlsx
+++ b/res/efficiency/pet-md/ollama-L3.3-MS-Nevoria-70b-Q4_K_S/2025-02-15_05-49-12/stats_by_iteration-L3.3-MS-Nevoria-70b-Q4_K_S.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="11">
   <si>
     <t>P</t>
   </si>
@@ -37,6 +37,12 @@
   </si>
   <si>
     <t>avg. power draw</t>
+  </si>
+  <si>
+    <t>output tokens</t>
+  </si>
+  <si>
+    <t>throughput</t>
   </si>
   <si>
     <t>parse_err</t>
@@ -494,10 +500,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -510,8 +516,14 @@
       <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4">
+      <c r="E1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>0.78133</v>
       </c>
@@ -524,8 +536,14 @@
       <c r="D2">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E2">
+        <v>50937</v>
+      </c>
+      <c r="F2">
+        <v>5.387878146816163</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>0.7778080000000001</v>
       </c>
@@ -538,8 +556,14 @@
       <c r="D3">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
+      <c r="E3">
+        <v>50673</v>
+      </c>
+      <c r="F3">
+        <v>5.393039591315453</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>0.66672</v>
       </c>
@@ -552,8 +576,14 @@
       <c r="D4">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="E4">
+        <v>48998</v>
+      </c>
+      <c r="F4">
+        <v>6.077648226246589</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>0.8409219999999999</v>
       </c>
@@ -566,8 +596,14 @@
       <c r="D5">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="E5">
+        <v>52574</v>
+      </c>
+      <c r="F5">
+        <v>5.17562512305572</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>0.718491</v>
       </c>
@@ -579,6 +615,12 @@
       </c>
       <c r="D6">
         <v>5</v>
+      </c>
+      <c r="E6">
+        <v>52984</v>
+      </c>
+      <c r="F6">
+        <v>6.102038465967984</v>
       </c>
     </row>
   </sheetData>
@@ -593,10 +635,10 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:2">

</xml_diff>